<commit_message>
Update kunnr_stats files and enhance country extraction logic
- Revised kunnr_stats.csv to reflect updated statistics with new country data.
- Modified count_kunnr_stats.py to include Australia and Brazil in the country mapping and added a new function to extract country codes from JSON data.
- Updated Excel file kunnr_stats.xlsx and various plot images to align with the latest data changes.
</commit_message>
<xml_diff>
--- a/app/kunnr_stats.xlsx
+++ b/app/kunnr_stats.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,25 +508,25 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>129079</v>
+        <v>5</v>
       </c>
       <c r="E2" t="n">
-        <v>77802</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>79819</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>62838</v>
+        <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>34296</v>
+        <v>4</v>
       </c>
       <c r="I2" t="n">
-        <v>60.3</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>61.8</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3">
@@ -537,12 +537,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Australia</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>8393</v>
+        <v>7</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -554,7 +554,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>8393</v>
+        <v>7</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -566,51 +566,51 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BE</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Belgium</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>365</v>
+        <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>365</v>
+        <v>0</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="J4" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>PL</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>11481</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>11481</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -634,17 +634,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CN</t>
+          <t>US</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>United States</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>4818</v>
+        <v>1</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>4818</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -668,371 +668,65 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>XX</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>55627</v>
+        <v>3</v>
       </c>
       <c r="E7" t="n">
-        <v>39808</v>
+        <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>40173</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>37008</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>12654</v>
+        <v>3</v>
       </c>
       <c r="I7" t="n">
-        <v>71.59999999999999</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>72.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>FR</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>France</t>
-        </is>
-      </c>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>124091</v>
+        <v>18</v>
       </c>
       <c r="E8" t="n">
-        <v>9160</v>
+        <v>1</v>
       </c>
       <c r="F8" t="n">
-        <v>11353</v>
+        <v>2</v>
       </c>
       <c r="G8" t="n">
-        <v>8094</v>
+        <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>111672</v>
+        <v>16</v>
       </c>
       <c r="I8" t="n">
-        <v>7.4</v>
+        <v>5.6</v>
       </c>
       <c r="J8" t="n">
-        <v>9.1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>MX</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="n">
-        <v>43791</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" t="n">
-        <v>43791</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>PL</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="n">
-        <v>47103</v>
-      </c>
-      <c r="E10" t="n">
-        <v>3914</v>
-      </c>
-      <c r="F10" t="n">
-        <v>791</v>
-      </c>
-      <c r="G10" t="n">
-        <v>97</v>
-      </c>
-      <c r="H10" t="n">
-        <v>42495</v>
-      </c>
-      <c r="I10" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="J10" t="n">
-        <v>1.7</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>RU</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="n">
-        <v>119707</v>
-      </c>
-      <c r="E11" t="n">
-        <v>500</v>
-      </c>
-      <c r="F11" t="n">
-        <v>85623</v>
-      </c>
-      <c r="G11" t="n">
-        <v>10</v>
-      </c>
-      <c r="H11" t="n">
-        <v>33594</v>
-      </c>
-      <c r="I11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="J11" t="n">
-        <v>71.5</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>TR</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Turkey</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="n">
-        <v>1027</v>
-      </c>
-      <c r="E12" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" t="n">
-        <v>0</v>
-      </c>
-      <c r="H12" t="n">
-        <v>1027</v>
-      </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>UA</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Ukraine</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="n">
-        <v>18069</v>
-      </c>
-      <c r="E13" t="n">
-        <v>14</v>
-      </c>
-      <c r="F13" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" t="n">
-        <v>4</v>
-      </c>
-      <c r="H13" t="n">
-        <v>18055</v>
-      </c>
-      <c r="I13" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>US</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>United States</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="n">
-        <v>94863</v>
-      </c>
-      <c r="E14" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" t="n">
-        <v>0</v>
-      </c>
-      <c r="H14" t="n">
-        <v>94863</v>
-      </c>
-      <c r="I14" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>XX</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="n">
-        <v>10</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" t="n">
-        <v>0</v>
-      </c>
-      <c r="H15" t="n">
-        <v>10</v>
-      </c>
-      <c r="I15" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>ZZ</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="n">
-        <v>80</v>
-      </c>
-      <c r="E16" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" t="n">
-        <v>66</v>
-      </c>
-      <c r="G16" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" t="n">
-        <v>14</v>
-      </c>
-      <c r="I16" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" t="n">
-        <v>82.5</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="n">
-        <v>658504</v>
-      </c>
-      <c r="E17" t="n">
-        <v>131198</v>
-      </c>
-      <c r="F17" t="n">
-        <v>217829</v>
-      </c>
-      <c r="G17" t="n">
-        <v>108051</v>
-      </c>
-      <c r="H17" t="n">
-        <v>417528</v>
-      </c>
-      <c r="I17" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="J17" t="n">
-        <v>33.1</v>
+        <v>11.1</v>
       </c>
     </row>
   </sheetData>
@@ -1114,25 +808,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>557638</v>
+        <v>7</v>
       </c>
       <c r="E2" t="n">
-        <v>118457</v>
+        <v>1</v>
       </c>
       <c r="F2" t="n">
-        <v>196738</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
-        <v>96628</v>
+        <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>339071</v>
+        <v>6</v>
       </c>
       <c r="I2" t="n">
-        <v>21.2</v>
+        <v>14.3</v>
       </c>
       <c r="J2" t="n">
-        <v>35.3</v>
+        <v>14.3</v>
       </c>
     </row>
     <row r="3">
@@ -1148,7 +842,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>16499</v>
+        <v>3</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -1160,7 +854,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>16499</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -1182,25 +876,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>84367</v>
+        <v>8</v>
       </c>
       <c r="E4" t="n">
-        <v>12741</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>21091</v>
+        <v>1</v>
       </c>
       <c r="G4" t="n">
-        <v>11423</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>61958</v>
+        <v>7</v>
       </c>
       <c r="I4" t="n">
-        <v>15.1</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>25</v>
+        <v>12.5</v>
       </c>
     </row>
     <row r="5">
@@ -1216,25 +910,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>658504</v>
+        <v>18</v>
       </c>
       <c r="E5" t="n">
-        <v>131198</v>
+        <v>1</v>
       </c>
       <c r="F5" t="n">
-        <v>217829</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
-        <v>108051</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>417528</v>
+        <v>16</v>
       </c>
       <c r="I5" t="n">
-        <v>19.9</v>
+        <v>5.6</v>
       </c>
       <c r="J5" t="n">
-        <v>33.1</v>
+        <v>11.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update kunnr_stats data with comprehensive country statistics and enhance visualizations
- Revised kunnr_stats.csv to include detailed statistics for multiple countries, versions, and new data points such as 'Missing' entries.
- Updated kunnr_stats.xlsx to reflect the latest changes in the CSV file.
- Modified various plot images to align with the updated statistics, ensuring accurate visual representation of the data.
- Enhanced summary sections in the CSV to provide a clearer overview of total counts and percentages across different categories.
</commit_message>
<xml_diff>
--- a/app/kunnr_stats.xlsx
+++ b/app/kunnr_stats.xlsx
@@ -440,7 +440,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -508,25 +508,25 @@
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>129079</v>
       </c>
       <c r="E2" t="n">
-        <v>0</v>
+        <v>77802</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>79819</v>
       </c>
       <c r="G2" t="n">
-        <v>0</v>
+        <v>62838</v>
       </c>
       <c r="H2" t="n">
-        <v>4</v>
+        <v>34296</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>60.3</v>
       </c>
       <c r="J2" t="n">
-        <v>20</v>
+        <v>61.8</v>
       </c>
     </row>
     <row r="3">
@@ -542,7 +542,7 @@
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>8400</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -554,7 +554,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>7</v>
+        <v>8400</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -566,51 +566,51 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>DE</t>
+          <t>BE</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Germany</t>
+          <t>Belgium</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>365</v>
       </c>
       <c r="E4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
+        <v>365</v>
       </c>
       <c r="I4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="J4" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PL</t>
+          <t>BR</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Brazil</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="n">
-        <v>1</v>
+        <v>11481</v>
       </c>
       <c r="E5" t="n">
         <v>0</v>
@@ -622,7 +622,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>1</v>
+        <v>11481</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -634,17 +634,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>US</t>
+          <t>CN</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>United States</t>
+          <t>China</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>4818</v>
       </c>
       <c r="E6" t="n">
         <v>0</v>
@@ -656,7 +656,7 @@
         <v>0</v>
       </c>
       <c r="H6" t="n">
-        <v>1</v>
+        <v>4818</v>
       </c>
       <c r="I6" t="n">
         <v>0</v>
@@ -668,65 +668,371 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>XX</t>
+          <t>DE</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Germany</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="n">
-        <v>3</v>
+        <v>55627</v>
       </c>
       <c r="E7" t="n">
-        <v>0</v>
+        <v>39808</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>40173</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>37008</v>
       </c>
       <c r="H7" t="n">
-        <v>3</v>
+        <v>12654</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ALL</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>FR</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>France</t>
+        </is>
+      </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="n">
-        <v>18</v>
+        <v>124091</v>
       </c>
       <c r="E8" t="n">
-        <v>1</v>
+        <v>9160</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>11353</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>8094</v>
       </c>
       <c r="H8" t="n">
-        <v>16</v>
+        <v>111672</v>
       </c>
       <c r="I8" t="n">
-        <v>5.6</v>
+        <v>7.4</v>
       </c>
       <c r="J8" t="n">
-        <v>11.1</v>
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>MX</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Mexico</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>43791</v>
+      </c>
+      <c r="E9" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="n">
+        <v>43791</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>PL</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>47103</v>
+      </c>
+      <c r="E10" t="n">
+        <v>3914</v>
+      </c>
+      <c r="F10" t="n">
+        <v>791</v>
+      </c>
+      <c r="G10" t="n">
+        <v>97</v>
+      </c>
+      <c r="H10" t="n">
+        <v>42495</v>
+      </c>
+      <c r="I10" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="J10" t="n">
+        <v>1.7</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>RU</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Russia</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>119707</v>
+      </c>
+      <c r="E11" t="n">
+        <v>500</v>
+      </c>
+      <c r="F11" t="n">
+        <v>85623</v>
+      </c>
+      <c r="G11" t="n">
+        <v>10</v>
+      </c>
+      <c r="H11" t="n">
+        <v>33594</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="J11" t="n">
+        <v>71.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>TR</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Turkey</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="n">
+        <v>1027</v>
+      </c>
+      <c r="E12" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1027</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>UA</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ukraine</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="n">
+        <v>18069</v>
+      </c>
+      <c r="E13" t="n">
+        <v>14</v>
+      </c>
+      <c r="F13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>4</v>
+      </c>
+      <c r="H13" t="n">
+        <v>18055</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="n">
+        <v>94863</v>
+      </c>
+      <c r="E14" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="n">
+        <v>94863</v>
+      </c>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>XX</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="n">
+        <v>3</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ZZ</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Custom / Unassigned</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="n">
+        <v>80</v>
+      </c>
+      <c r="E16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" t="n">
+        <v>66</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="n">
+        <v>14</v>
+      </c>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>82.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>ALL</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="n">
+        <v>658504</v>
+      </c>
+      <c r="E17" t="n">
+        <v>131198</v>
+      </c>
+      <c r="F17" t="n">
+        <v>217829</v>
+      </c>
+      <c r="G17" t="n">
+        <v>108051</v>
+      </c>
+      <c r="H17" t="n">
+        <v>417528</v>
+      </c>
+      <c r="I17" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="J17" t="n">
+        <v>33.1</v>
       </c>
     </row>
   </sheetData>
@@ -808,25 +1114,25 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>7</v>
+        <v>557638</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>118457</v>
       </c>
       <c r="F2" t="n">
-        <v>1</v>
+        <v>196738</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>96628</v>
       </c>
       <c r="H2" t="n">
-        <v>6</v>
+        <v>339071</v>
       </c>
       <c r="I2" t="n">
-        <v>14.3</v>
+        <v>21.2</v>
       </c>
       <c r="J2" t="n">
-        <v>14.3</v>
+        <v>35.3</v>
       </c>
     </row>
     <row r="3">
@@ -842,7 +1148,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>3</v>
+        <v>16499</v>
       </c>
       <c r="E3" t="n">
         <v>0</v>
@@ -854,7 +1160,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>16499</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -876,25 +1182,25 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>8</v>
+        <v>84367</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>12741</v>
       </c>
       <c r="F4" t="n">
-        <v>1</v>
+        <v>21091</v>
       </c>
       <c r="G4" t="n">
-        <v>0</v>
+        <v>11423</v>
       </c>
       <c r="H4" t="n">
-        <v>7</v>
+        <v>61958</v>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>15.1</v>
       </c>
       <c r="J4" t="n">
-        <v>12.5</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5">
@@ -910,25 +1216,25 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>18</v>
+        <v>658504</v>
       </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>131198</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>217829</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>108051</v>
       </c>
       <c r="H5" t="n">
-        <v>16</v>
+        <v>417528</v>
       </c>
       <c r="I5" t="n">
-        <v>5.6</v>
+        <v>19.9</v>
       </c>
       <c r="J5" t="n">
-        <v>11.1</v>
+        <v>33.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>